<commit_message>
actualisation tableau de synthèse
</commit_message>
<xml_diff>
--- a/tableau_synthese.xlsx
+++ b/tableau_synthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julien\Documents\BTS SIO Iris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AEA077-B15E-404E-8EB5-0D33C37D9D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68FA4F9B-B65C-4A0F-8852-FD7EB3592D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -166,6 +166,31 @@
   </si>
   <si>
     <t>Adresse URL du portfolio : https://julienmarcucci.github.io/Portfolio/</t>
+  </si>
+  <si>
+    <t>Câblage pour relier les prises réseau au switch</t>
+  </si>
+  <si>
+    <t>Inventaire du matériel informatique existant de l'entreprise ainsi que le nouveau</t>
+  </si>
+  <si>
+    <t>Travail en autonomie sur des notions informatiques : Windows Server, protocole TCP/IP. Je me
+suis renseigné sur le métier de technicien informatique.</t>
+  </si>
+  <si>
+    <t>Réalisation de tests de connectivité et de performance réseau (ping, speed test)</t>
+  </si>
+  <si>
+    <t>Identification du matériel informatique, schématiser l'infrastructure pour avoir une vue d'ensemble</t>
+  </si>
+  <si>
+    <t>Étude du fonctionnement du logiciel HelloDoc puis audit et amélioration de la politique de sauvegarde des données médicales dans le respect du RGPD</t>
+  </si>
+  <si>
+    <t>Proposition de mise en place d'un trousseau de mots de passe pour générer des mots de passe sécurisés et les stocker</t>
+  </si>
+  <si>
+    <t>Support informatique et assistance aux utilisateurs</t>
   </si>
 </sst>
 </file>
@@ -737,9 +762,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -762,45 +826,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1185,56 +1210,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="24"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="31" t="s">
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="32"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="45"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="12" t="s">
         <v>2</v>
       </c>
@@ -1246,22 +1271,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="33" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1284,8 +1309,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="42"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
@@ -1341,16 +1366,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="29"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1811,16 +1836,16 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="40"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="32"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1858,7 +1883,9 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
+      <c r="A19" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="B19" s="8"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
@@ -1903,7 +1930,9 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
+      <c r="A20" s="9" t="s">
+        <v>37</v>
+      </c>
       <c r="B20" s="8"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
@@ -1948,7 +1977,9 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
+      <c r="A21" s="9" t="s">
+        <v>38</v>
+      </c>
       <c r="B21" s="8"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
@@ -2173,16 +2204,16 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="40"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="32"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2220,7 +2251,9 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
+      <c r="A27" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="B27" s="8"/>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
@@ -2265,7 +2298,9 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="9"/>
+      <c r="A28" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="B28" s="8"/>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
@@ -2310,7 +2345,9 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
+      <c r="A29" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="B29" s="8"/>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
@@ -2355,7 +2392,9 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
+      <c r="A30" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="B30" s="8"/>
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
@@ -2400,7 +2439,9 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
+      <c r="A31" s="9" t="s">
+        <v>43</v>
+      </c>
       <c r="B31" s="8"/>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
@@ -2627,6 +2668,11 @@
     <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2634,11 +2680,6 @@
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2650,12 +2691,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="665588ff-5dd3-431a-aaf4-bd4a76d54561">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8dfcfa40-b15b-4f0f-a13d-24527312d446" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2866,20 +2909,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="665588ff-5dd3-431a-aaf4-bd4a76d54561">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8dfcfa40-b15b-4f0f-a13d-24527312d446" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A9CD917-9C6C-4808-B3EB-08BF761FD3DB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B48EC0E1-0992-4BEA-AB73-03077E430CDC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="665588ff-5dd3-431a-aaf4-bd4a76d54561"/>
+    <ds:schemaRef ds:uri="8dfcfa40-b15b-4f0f-a13d-24527312d446"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2904,12 +2948,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B48EC0E1-0992-4BEA-AB73-03077E430CDC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A9CD917-9C6C-4808-B3EB-08BF761FD3DB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="665588ff-5dd3-431a-aaf4-bd4a76d54561"/>
-    <ds:schemaRef ds:uri="8dfcfa40-b15b-4f0f-a13d-24527312d446"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>